<commit_message>
atualiza volumes loa com ppo - 03092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_REPASSE_RECURSOS.xlsx
+++ b/bancos/SISOR/BASE_REPASSE_RECURSOS.xlsx
@@ -464,92 +464,92 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1011</v>
+        <v>4711</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1501</v>
+        <v>1091</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>PROCURADORIA GERAL DE JUSTIÇA</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>103231</v>
+        <v>300411652</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1301</v>
+        <v>4711</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIAS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4631</v>
+        <v>1091</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FUNDO DE PAGAMENTO DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
+          <t>PROCURADORIA GERAL DE JUSTIÇA</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>3372264</v>
+        <v>448050447</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2011</v>
+        <v>4381</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1501</v>
+        <v>1191</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>SECRETARIA DE ESTADO DE FAZENDA</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
@@ -558,214 +558,214 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>6980303</v>
+        <v>1008000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2011</v>
+        <v>4711</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1941</v>
+        <v>1021</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EGE-SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>TRIBUNAL DE CONTAS DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>100000</v>
+        <v>133292078</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2041</v>
+        <v>4711</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LOTERIA DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1501</v>
+        <v>1021</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>TRIBUNAL DE CONTAS DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>307920</v>
+        <v>115233552</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2041</v>
+        <v>4711</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LOTERIA DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4711</v>
+        <v>1051</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>TRIBUNAL DE JUSTIÇA MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>1776827</v>
+        <v>8800648</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2071</v>
+        <v>4711</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO DE AMPARO À PESQUISA DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4711</v>
+        <v>1051</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>TRIBUNAL DE JUSTIÇA MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>16838</v>
+        <v>11045990</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2091</v>
+        <v>4711</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1371</v>
+        <v>1011</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE MEIO AMBIENTE E DESENVOLVIMENTO SUSTENTÁVEL</t>
+          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>13000000</v>
+        <v>129510000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2091</v>
+        <v>4711</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1501</v>
+        <v>1011</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1633636</v>
+        <v>120000000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2091</v>
+        <v>2261</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
+          <t>FUNDAÇÃO EZEQUIEL DIAS</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -780,7 +780,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
@@ -789,31 +789,31 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>4859876</v>
+        <v>34739894</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2101</v>
+        <v>1301</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>INSTITUTO ESTADUAL DE FLORESTAS</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIAS</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1401</v>
+        <v>4631</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CORPO DE BOMBEIROS MILITAR DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO DE PAGAMENTO DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G12" t="n">
         <v>2</v>
@@ -822,28 +822,28 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>6682057</v>
+        <v>727000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2101</v>
+        <v>4381</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>INSTITUTO ESTADUAL DE FLORESTAS</t>
+          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1501</v>
+        <v>2471</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>AGÊNCIA REGULADORA DE TRANSPORTES DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
         <v>60</v>
@@ -855,24 +855,24 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>2015107</v>
+        <v>17964220</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2101</v>
+        <v>4381</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>INSTITUTO ESTADUAL DE FLORESTAS</t>
+          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4031</v>
+        <v>2471</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FUNDO ESPECIAL DO PODER JUDICIÁRIO DO ESTADO DE MINAS GERAIS</t>
+          <t>AGÊNCIA REGULADORA DE TRANSPORTES DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -888,31 +888,31 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>120000</v>
+        <v>5780000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2121</v>
+        <v>2371</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES MILITARES DO ESTADO DE MINAS GERAIS</t>
+          <t>INSTITUTO MINEIRO DE AGROPECUÁRIA</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1251</v>
+        <v>1501</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G15" t="n">
         <v>2</v>
@@ -921,28 +921,28 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>134472993</v>
+        <v>149161</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2121</v>
+        <v>2091</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES MILITARES DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1251</v>
+        <v>4711</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>60</v>
@@ -954,7 +954,7 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>9754107</v>
+        <v>155090</v>
       </c>
     </row>
     <row r="17">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
         <v>60</v>
@@ -987,7 +987,7 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>822699</v>
+        <v>575076</v>
       </c>
     </row>
     <row r="18">
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>60</v>
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>48202</v>
+        <v>1004919</v>
       </c>
     </row>
     <row r="19">
@@ -1033,18 +1033,18 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1501</v>
+        <v>1251</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
+          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -1053,7 +1053,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>12444</v>
+        <v>15642001</v>
       </c>
     </row>
     <row r="20">
@@ -1066,18 +1066,18 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4711</v>
+        <v>1251</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -1086,16 +1086,16 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>884722</v>
+        <v>140778004</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2241</v>
+        <v>2121</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>INSTITUTO MINEIRO DE GESTÃO DAS ÁGUAS</t>
+          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES MILITARES DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1119,31 +1119,31 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>1381549</v>
+        <v>107449</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2251</v>
+        <v>2091</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>JUNTA COMERCIAL DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4711</v>
+        <v>1501</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G22" t="n">
         <v>2</v>
@@ -1152,31 +1152,31 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>4207639</v>
+        <v>2177178</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2261</v>
+        <v>2091</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO EZEQUIEL DIAS</t>
+          <t>FUNDAÇÃO ESTADUAL DO MEIO AMBIENTE</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4711</v>
+        <v>1371</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE MEIO AMBIENTE E DESENVOLVIMENTO SUSTENTÁVEL</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="G23" t="n">
         <v>2</v>
@@ -1185,31 +1185,31 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>32737210</v>
+        <v>13650000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2271</v>
+        <v>2241</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO HOSPITALAR DO ESTADO DE MINAS GERAIS</t>
+          <t>INSTITUTO MINEIRO DE GESTÃO DAS ÁGUAS</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4711</v>
+        <v>1501</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G24" t="n">
         <v>2</v>
@@ -1218,16 +1218,16 @@
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>235218509</v>
+        <v>1774713</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2321</v>
+        <v>2041</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO CENTRO DE HEMATOLOGIA E HEMOTERAPIA DE MINAS GERAIS</t>
+          <t>LOTERIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1251,16 +1251,16 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>27341045</v>
+        <v>1686000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2371</v>
+        <v>2041</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>INSTITUTO MINEIRO DE AGROPECUÁRIA</t>
+          <t>LOTERIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1275,7 +1275,7 @@
         <v>3</v>
       </c>
       <c r="F26" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="G26" t="n">
         <v>2</v>
@@ -1284,7 +1284,7 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>221046</v>
+        <v>458582</v>
       </c>
     </row>
     <row r="27">
@@ -1317,28 +1317,28 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>1290973</v>
+        <v>1707737</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>4031</v>
+        <v>2251</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FUNDO ESPECIAL DO PODER JUDICIÁRIO DO ESTADO DE MINAS GERAIS</t>
+          <t>JUNTA COMERCIAL DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1451</v>
+        <v>4711</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE JUSTIÇA E SEGURANÇA PÚBLICA</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>60</v>
@@ -1350,28 +1350,28 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>875221853</v>
+        <v>4444845</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>4031</v>
+        <v>2321</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>FUNDO ESPECIAL DO PODER JUDICIÁRIO DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDAÇÃO CENTRO DE HEMATOLOGIA E HEMOTERAPIA DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1451</v>
+        <v>4711</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE JUSTIÇA E SEGURANÇA PÚBLICA</t>
+          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
         <v>60</v>
@@ -1380,19 +1380,19 @@
         <v>2</v>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>1778147</v>
+        <v>31836274</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4031</v>
+        <v>2101</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>FUNDO ESPECIAL DO PODER JUDICIÁRIO DO ESTADO DE MINAS GERAIS</t>
+          <t>INSTITUTO ESTADUAL DE FLORESTAS</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1407,7 +1407,7 @@
         <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G30" t="n">
         <v>2</v>
@@ -1416,31 +1416,31 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>1318193</v>
+        <v>3110043</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4111</v>
+        <v>4031</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>FUNDO DE FOMENTO E DESENVOLVIMENTO SOCIOECONÔMICO DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO ESPECIAL DO PODER JUDICIÁRIO DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1915</v>
+        <v>1501</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>PARTICIPAÇÃO NO AUMENTO DO CAPITAL SOCIAL DE EMPRESAS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G31" t="n">
         <v>2</v>
@@ -1449,31 +1449,31 @@
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>110000</v>
+        <v>1570548</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>4291</v>
+        <v>4031</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE SAÚDE</t>
+          <t>FUNDO ESPECIAL DO PODER JUDICIÁRIO DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1451</v>
+        <v>1081</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE JUSTIÇA E SEGURANÇA PÚBLICA</t>
+          <t>ADVOCACIA GERAL DO ESTADO</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G32" t="n">
         <v>2</v>
@@ -1482,31 +1482,31 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>1138967</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>4291</v>
+        <v>4381</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE SAÚDE</t>
+          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1511</v>
+        <v>1251</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>POLÍCIA CIVIL DO ESTADO DE MINAS GERAIS</t>
+          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="G33" t="n">
         <v>2</v>
@@ -1515,64 +1515,64 @@
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>13543</v>
+        <v>15000000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>4291</v>
+        <v>1271</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE SAÚDE</t>
+          <t>SECRETARIA DE ESTADO DE CULTURA E TURISMO</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2011</v>
+        <v>4491</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES DO ESTADO DE MINAS GERAIS</t>
+          <t>FUNDO ESTADUAL DE CULTURA</t>
         </is>
       </c>
       <c r="E34" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>16</v>
+      </c>
+      <c r="G34" t="n">
         <v>1</v>
       </c>
-      <c r="F34" t="n">
-        <v>57</v>
-      </c>
-      <c r="G34" t="n">
-        <v>2</v>
-      </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>7356625</v>
+        <v>130003000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>4291</v>
+        <v>2011</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE SAÚDE</t>
+          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2121</v>
+        <v>1941</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES MILITARES DO ESTADO DE MINAS GERAIS</t>
+          <t>EGE-SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -1581,31 +1581,31 @@
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>70000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>4291</v>
+        <v>2011</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE SAÚDE</t>
+          <t>INSTITUTO DE PREVIDÊNCIA DOS SERVIDORES DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2261</v>
+        <v>1501</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO EZEQUIEL DIAS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G36" t="n">
         <v>2</v>
@@ -1614,31 +1614,31 @@
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>13845</v>
+        <v>6311890</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>4291</v>
+        <v>1011</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE SAÚDE</t>
+          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2271</v>
+        <v>1501</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO HOSPITALAR DO ESTADO DE MINAS GERAIS</t>
+          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G37" t="n">
         <v>2</v>
@@ -1647,31 +1647,31 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>32667892</v>
+        <v>104706</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>4291</v>
+        <v>4111</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE SAÚDE</t>
+          <t>FUNDO DE FOMENTO E DESENVOLVIMENTO SOCIOECONÔMICO DO ESTADO DE MINAS GERAIS</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2311</v>
+        <v>1915</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>UNIVERSIDADE ESTADUAL DE MONTES CLAROS</t>
+          <t>PARTICIPAÇÃO NO AUMENTO DO CAPITAL SOCIAL DE EMPRESAS</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F38" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
@@ -1680,634 +1680,7 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>1794000</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>4291</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>FUNDO ESTADUAL DE SAÚDE</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>2321</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>FUNDAÇÃO CENTRO DE HEMATOLOGIA E HEMOTERAPIA DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" t="n">
-        <v>57</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>780000</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>4381</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>1191</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE FAZENDA</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>3</v>
-      </c>
-      <c r="F40" t="n">
-        <v>83</v>
-      </c>
-      <c r="G40" t="n">
-        <v>2</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" t="n">
-        <v>960000</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>4381</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>1251</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>POLÍCIA MILITAR DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>3</v>
-      </c>
-      <c r="F41" t="n">
-        <v>83</v>
-      </c>
-      <c r="G41" t="n">
-        <v>2</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" t="n">
-        <v>15000000</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>4381</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>2471</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>AGÊNCIA REGULADORA DE TRANSPORTES DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>3</v>
-      </c>
-      <c r="F42" t="n">
-        <v>60</v>
-      </c>
-      <c r="G42" t="n">
-        <v>2</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" t="n">
-        <v>2001130</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>4381</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>2471</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>AGÊNCIA REGULADORA DE TRANSPORTES DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>4</v>
-      </c>
-      <c r="F43" t="n">
-        <v>60</v>
-      </c>
-      <c r="G43" t="n">
-        <v>2</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>37635820</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>4381</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>4631</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>FUNDO DE PAGAMENTO DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>5</v>
-      </c>
-      <c r="F44" t="n">
-        <v>60</v>
-      </c>
-      <c r="G44" t="n">
-        <v>2</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" t="n">
-        <v>60788935</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>4491</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>FUNDO ESTADUAL DE CULTURA</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>3151</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>EMPRESA MINEIRA DE COMUNICAÇÃO</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>3</v>
-      </c>
-      <c r="F45" t="n">
-        <v>59</v>
-      </c>
-      <c r="G45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H45" t="n">
-        <v>1</v>
-      </c>
-      <c r="I45" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>1011</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" t="n">
-        <v>43</v>
-      </c>
-      <c r="G46" t="n">
-        <v>5</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0</v>
-      </c>
-      <c r="I46" t="n">
-        <v>126400000</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>1011</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" t="n">
-        <v>42</v>
-      </c>
-      <c r="G47" t="n">
-        <v>5</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>112000000</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>1021</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>TRIBUNAL DE CONTAS DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" t="n">
-        <v>42</v>
-      </c>
-      <c r="G48" t="n">
-        <v>5</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" t="n">
-        <v>104407495</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>1021</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>TRIBUNAL DE CONTAS DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" t="n">
-        <v>43</v>
-      </c>
-      <c r="G49" t="n">
-        <v>5</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" t="n">
-        <v>118906754</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>1031</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>TRIBUNAL DE JUSTIÇA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" t="n">
-        <v>43</v>
-      </c>
-      <c r="G50" t="n">
-        <v>5</v>
-      </c>
-      <c r="H50" t="n">
-        <v>0</v>
-      </c>
-      <c r="I50" t="n">
-        <v>891570030</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>1031</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>TRIBUNAL DE JUSTIÇA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" t="n">
-        <v>42</v>
-      </c>
-      <c r="G51" t="n">
-        <v>5</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0</v>
-      </c>
-      <c r="I51" t="n">
-        <v>1081813774</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>1051</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>TRIBUNAL DE JUSTIÇA MILITAR DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" t="n">
-        <v>43</v>
-      </c>
-      <c r="G52" t="n">
-        <v>5</v>
-      </c>
-      <c r="H52" t="n">
-        <v>0</v>
-      </c>
-      <c r="I52" t="n">
-        <v>9665367</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>1051</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>TRIBUNAL DE JUSTIÇA MILITAR DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" t="n">
-        <v>42</v>
-      </c>
-      <c r="G53" t="n">
-        <v>5</v>
-      </c>
-      <c r="H53" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" t="n">
-        <v>9851943</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>1091</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>PROCURADORIA GERAL DE JUSTIÇA</t>
-        </is>
-      </c>
-      <c r="E54" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" t="n">
-        <v>42</v>
-      </c>
-      <c r="G54" t="n">
-        <v>5</v>
-      </c>
-      <c r="H54" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" t="n">
-        <v>391082727</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>1091</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>PROCURADORIA GERAL DE JUSTIÇA</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" t="n">
-        <v>43</v>
-      </c>
-      <c r="G55" t="n">
-        <v>5</v>
-      </c>
-      <c r="H55" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" t="n">
-        <v>260748891</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>1441</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>DEFENSORIA PUBLICA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E56" t="n">
-        <v>1</v>
-      </c>
-      <c r="F56" t="n">
-        <v>42</v>
-      </c>
-      <c r="G56" t="n">
-        <v>5</v>
-      </c>
-      <c r="H56" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" t="n">
-        <v>101210335</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>4711</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>FUNDO FINANCEIRO DE PREVIDÊNCIA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>1441</v>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>DEFENSORIA PUBLICA DO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>1</v>
-      </c>
-      <c r="F57" t="n">
-        <v>43</v>
-      </c>
-      <c r="G57" t="n">
-        <v>5</v>
-      </c>
-      <c r="H57" t="n">
-        <v>0</v>
-      </c>
-      <c r="I57" t="n">
-        <v>67978647</v>
+        <v>98000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>